<commit_message>
compile_tigress.py now uses the randomized seed.
extract_ngrams.py now traverses the randomized tigress binaries.

gen_plots.py now computes the answers to rq2 and 3.

validate.py now tests the tigress binaries produced by randomized seed
</commit_message>
<xml_diff>
--- a/jsd_results.xlsx
+++ b/jsd_results.xlsx
@@ -5197,67 +5197,67 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4595860889341547</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4740875357356574</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4753285233614369</v>
       </c>
       <c r="E2" t="n">
-        <v>0.499645410718047</v>
+        <v>0.499277873098543</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4898151799500335</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4928870198107494</v>
       </c>
       <c r="H2" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5161041678862056</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5009720722564039</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5110663418013732</v>
       </c>
       <c r="K2" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4619574927513915</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4771225483488299</v>
       </c>
       <c r="M2" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4708984051478177</v>
       </c>
       <c r="N2" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4911005652488126</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4634478735784001</v>
       </c>
       <c r="P2" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4856236667399766</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4826245294492603</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.494267440249476</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5126403230067331</v>
       </c>
       <c r="T2" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4822973951538623</v>
       </c>
       <c r="U2" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5057738959478034</v>
       </c>
       <c r="V2" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4945876589007914</v>
       </c>
     </row>
     <row r="3">
@@ -5267,67 +5267,67 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4677449200831341</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4863633719629789</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4734653657383854</v>
       </c>
       <c r="E3" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4926350351616487</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.483166872883638</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4938781083123851</v>
       </c>
       <c r="H3" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5123231388086434</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4948425768806</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5018108367229078</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4765925326592631</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4773330605927134</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4701560500585655</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.485759493220699</v>
       </c>
       <c r="O3" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4611737360708684</v>
       </c>
       <c r="P3" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4759669233481278</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4719828207925485</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4939531680948803</v>
       </c>
       <c r="S3" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5068986377262799</v>
       </c>
       <c r="T3" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4796327872535199</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5013795468178642</v>
       </c>
       <c r="V3" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4987335984562077</v>
       </c>
     </row>
     <row r="4">
@@ -5337,67 +5337,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4718176364020177</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4837702261121167</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4759025586747268</v>
       </c>
       <c r="E4" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4996087791969133</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4859602243348099</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4915190210598347</v>
       </c>
       <c r="H4" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5114784808366629</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5011945307572392</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5095029931304007</v>
       </c>
       <c r="K4" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4628050257036362</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4846257621526322</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4802117314713114</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4835332864912293</v>
       </c>
       <c r="O4" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4624519334526769</v>
       </c>
       <c r="P4" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4903617005020591</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4862916287970999</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.483690056120035</v>
       </c>
       <c r="S4" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5092591418003439</v>
       </c>
       <c r="T4" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4824633797510544</v>
       </c>
       <c r="U4" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.4974087712129504</v>
       </c>
       <c r="V4" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4931319962266868</v>
       </c>
     </row>
     <row r="5">
@@ -5407,67 +5407,67 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4774509804463585</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4792516893855388</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4861408483928702</v>
       </c>
       <c r="E5" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4907679543021317</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4941222870561732</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.5006989637651839</v>
       </c>
       <c r="H5" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5112099552823521</v>
       </c>
       <c r="I5" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5009413793240323</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5113736700344444</v>
       </c>
       <c r="K5" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4566571433352663</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4782963801854045</v>
       </c>
       <c r="M5" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4761941256769107</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4864107797009606</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4601478535120703</v>
       </c>
       <c r="P5" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4841540969157127</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4832207198035355</v>
       </c>
       <c r="R5" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.49046464881866</v>
       </c>
       <c r="S5" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5003384529952489</v>
       </c>
       <c r="T5" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4813309963645223</v>
       </c>
       <c r="U5" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.4987951050074856</v>
       </c>
       <c r="V5" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4965834431598432</v>
       </c>
     </row>
     <row r="6">
@@ -5477,67 +5477,67 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4818328161290666</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4772840173899592</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4651960518798533</v>
       </c>
       <c r="E6" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4946548277905271</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4984082085148288</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4929162788435474</v>
       </c>
       <c r="H6" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5125857047454022</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5002206686970105</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5001124234642015</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4632956926074455</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4765543471987593</v>
       </c>
       <c r="M6" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4650642260006001</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.488640432494674</v>
       </c>
       <c r="O6" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.456547645871892</v>
       </c>
       <c r="P6" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4906465529613461</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4829725790442145</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.5015817821914492</v>
       </c>
       <c r="S6" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5065805371637988</v>
       </c>
       <c r="T6" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4794065337346239</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.4988227195726322</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4981992720298212</v>
       </c>
     </row>
     <row r="7">
@@ -5547,67 +5547,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4738378531638212</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4755060629750529</v>
       </c>
       <c r="D7" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4798658945810579</v>
       </c>
       <c r="E7" t="n">
-        <v>0.499645410718047</v>
+        <v>0.500697332570393</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4896549951470634</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4981981291669912</v>
       </c>
       <c r="H7" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5061635464967881</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4948250877301242</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5114283994299555</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4645639681445281</v>
       </c>
       <c r="L7" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4817095385591108</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4693149170078822</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4921011405067843</v>
       </c>
       <c r="O7" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4538493100920224</v>
       </c>
       <c r="P7" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4827104686564206</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4898593950140167</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.488252142373571</v>
       </c>
       <c r="S7" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5104448756407264</v>
       </c>
       <c r="T7" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.477315647468619</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5074167707750853</v>
       </c>
       <c r="V7" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4968714578335715</v>
       </c>
     </row>
     <row r="8">
@@ -5617,67 +5617,67 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4718766199151857</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.482609431560395</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4675729190397862</v>
       </c>
       <c r="E8" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4977311545993031</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4871894612802555</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4931203851243935</v>
       </c>
       <c r="H8" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5058462478480925</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4933193163451077</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.517342282049521</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4627983625650877</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4715588888561162</v>
       </c>
       <c r="M8" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.465568235874691</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4848776345201585</v>
       </c>
       <c r="O8" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4640623870418119</v>
       </c>
       <c r="P8" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4867556297439275</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4895210349212166</v>
       </c>
       <c r="R8" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4885560066719007</v>
       </c>
       <c r="S8" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5076167990600148</v>
       </c>
       <c r="T8" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4840621711308415</v>
       </c>
       <c r="U8" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5001649904738489</v>
       </c>
       <c r="V8" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4939684973786773</v>
       </c>
     </row>
     <row r="9">
@@ -5687,67 +5687,67 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4697551012028731</v>
       </c>
       <c r="C9" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4765304198799364</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4716815791646639</v>
       </c>
       <c r="E9" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4917216845728802</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4773645190399252</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4949366712411519</v>
       </c>
       <c r="H9" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5038357329042576</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.500905698501099</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5098877891517538</v>
       </c>
       <c r="K9" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.478511600364548</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4891529488052719</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4721736781879833</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4955707499768895</v>
       </c>
       <c r="O9" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4555015053159098</v>
       </c>
       <c r="P9" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4918749581838399</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4844215132321317</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4957375676385019</v>
       </c>
       <c r="S9" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5050101872539594</v>
       </c>
       <c r="T9" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4854894322007713</v>
       </c>
       <c r="U9" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.4994365532873558</v>
       </c>
       <c r="V9" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4907734373078683</v>
       </c>
     </row>
     <row r="10">
@@ -5757,67 +5757,67 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4779959025286734</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4736966196212902</v>
       </c>
       <c r="D10" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4729000086580042</v>
       </c>
       <c r="E10" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4949476249717899</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.486899438893007</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4931822455265678</v>
       </c>
       <c r="H10" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5083972417486827</v>
       </c>
       <c r="I10" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5018215066140924</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5047163658172655</v>
       </c>
       <c r="K10" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4555690502078079</v>
       </c>
       <c r="L10" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4716394299439224</v>
       </c>
       <c r="M10" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4720090665309948</v>
       </c>
       <c r="N10" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4887735745216073</v>
       </c>
       <c r="O10" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.458698916015667</v>
       </c>
       <c r="P10" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4810375297160949</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4869535577331774</v>
       </c>
       <c r="R10" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4927663909978506</v>
       </c>
       <c r="S10" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5091612981393119</v>
       </c>
       <c r="T10" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4796045582187937</v>
       </c>
       <c r="U10" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5007016342027754</v>
       </c>
       <c r="V10" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4908170775151202</v>
       </c>
     </row>
     <row r="11">
@@ -5827,67 +5827,67 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.470452888438528</v>
+        <v>0.474075181916214</v>
       </c>
       <c r="C11" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4703518295428357</v>
       </c>
       <c r="D11" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4789690695697479</v>
       </c>
       <c r="E11" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4958573116610155</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4848600194042639</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4889708855178317</v>
       </c>
       <c r="H11" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5126851863656342</v>
       </c>
       <c r="I11" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4890348552997656</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5117880278058228</v>
       </c>
       <c r="K11" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4691400827658957</v>
       </c>
       <c r="L11" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4812092851478537</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4680264478616065</v>
       </c>
       <c r="N11" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4955621080650711</v>
       </c>
       <c r="O11" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4635694795817089</v>
       </c>
       <c r="P11" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4766941252367173</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4900870591310111</v>
       </c>
       <c r="R11" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4934020152710372</v>
       </c>
       <c r="S11" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5055332602111142</v>
       </c>
       <c r="T11" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4803455632250275</v>
       </c>
       <c r="U11" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5022043812794668</v>
       </c>
       <c r="V11" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4987309880186005</v>
       </c>
     </row>
     <row r="12">
@@ -5897,67 +5897,67 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.470452888438528</v>
+        <v>0.476318761767099</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4748575424940448</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4757723829038174</v>
       </c>
       <c r="E12" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4925387708266824</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4940131732223629</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4873506791027883</v>
       </c>
       <c r="H12" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5084510315910128</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4957019700281794</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5083316750200572</v>
       </c>
       <c r="K12" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4766724147260509</v>
       </c>
       <c r="L12" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4801966709870459</v>
       </c>
       <c r="M12" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4600894324226448</v>
       </c>
       <c r="N12" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4947844586400565</v>
       </c>
       <c r="O12" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.458490597302052</v>
       </c>
       <c r="P12" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4778753574176027</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4848940191339222</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4887271471439104</v>
       </c>
       <c r="S12" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5049757450279255</v>
       </c>
       <c r="T12" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4912758716435102</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5044981588870425</v>
       </c>
       <c r="V12" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.5009879556511679</v>
       </c>
     </row>
     <row r="13">
@@ -5967,67 +5967,67 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4824265498812263</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.47563399373276</v>
       </c>
       <c r="D13" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4826573173243868</v>
       </c>
       <c r="E13" t="n">
-        <v>0.499645410718047</v>
+        <v>0.496446917564849</v>
       </c>
       <c r="F13" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4827364923943789</v>
       </c>
       <c r="G13" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4927757915167027</v>
       </c>
       <c r="H13" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5020403669654103</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.5039575050791865</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5097828431426853</v>
       </c>
       <c r="K13" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4741876154525027</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4832982120994322</v>
       </c>
       <c r="M13" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4653642404389194</v>
       </c>
       <c r="N13" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4847532747274976</v>
       </c>
       <c r="O13" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4617839682336897</v>
       </c>
       <c r="P13" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4795018702507444</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4781993396862412</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.486340299536633</v>
       </c>
       <c r="S13" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5074411041436842</v>
       </c>
       <c r="T13" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.478087836084739</v>
       </c>
       <c r="U13" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5034382997475363</v>
       </c>
       <c r="V13" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.491477648784349</v>
       </c>
     </row>
     <row r="14">
@@ -6037,67 +6037,67 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4803885998659242</v>
       </c>
       <c r="C14" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4754570525562467</v>
       </c>
       <c r="D14" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.476495789633873</v>
       </c>
       <c r="E14" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4975013216448256</v>
       </c>
       <c r="F14" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4831953039896082</v>
       </c>
       <c r="G14" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4880290843646621</v>
       </c>
       <c r="H14" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5089009923877081</v>
       </c>
       <c r="I14" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.496626000145947</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5067169808440635</v>
       </c>
       <c r="K14" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4696517168960469</v>
       </c>
       <c r="L14" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4778083801561591</v>
       </c>
       <c r="M14" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.466486536738463</v>
       </c>
       <c r="N14" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.484320030699006</v>
       </c>
       <c r="O14" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4493150250214304</v>
       </c>
       <c r="P14" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4796071126276182</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4800804277041585</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4902005822822381</v>
       </c>
       <c r="S14" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5074250226582518</v>
       </c>
       <c r="T14" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4797675914546405</v>
       </c>
       <c r="U14" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.490263985610301</v>
       </c>
       <c r="V14" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4977789999771004</v>
       </c>
     </row>
     <row r="15">
@@ -6107,67 +6107,67 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4762944064595922</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4732732000398473</v>
       </c>
       <c r="D15" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4779497615249546</v>
       </c>
       <c r="E15" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4982830612137194</v>
       </c>
       <c r="F15" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4891429444661765</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.486395878018962</v>
       </c>
       <c r="H15" t="n">
-        <v>0.511631189803649</v>
+        <v>0.5048028971110061</v>
       </c>
       <c r="I15" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4956957934007378</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5092229323589663</v>
       </c>
       <c r="K15" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4572337393082131</v>
       </c>
       <c r="L15" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4856803153929254</v>
       </c>
       <c r="M15" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4758985862357056</v>
       </c>
       <c r="N15" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4836759312345058</v>
       </c>
       <c r="O15" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4636489139981455</v>
       </c>
       <c r="P15" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4853299071370194</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4894271767462116</v>
       </c>
       <c r="R15" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4934711712317155</v>
       </c>
       <c r="S15" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5068686375001262</v>
       </c>
       <c r="T15" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4844288679923385</v>
       </c>
       <c r="U15" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5099607270392688</v>
       </c>
       <c r="V15" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4986073949807795</v>
       </c>
     </row>
     <row r="16">
@@ -6177,67 +6177,67 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.470452888438528</v>
+        <v>0.480091074522849</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4751403808187614</v>
       </c>
       <c r="D16" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4779862889829244</v>
       </c>
       <c r="E16" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4939047516129775</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4896822127964206</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4936390349003515</v>
       </c>
       <c r="H16" t="n">
-        <v>0.511631189803649</v>
+        <v>0.4994013289819083</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4962594016625904</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5061516588212266</v>
       </c>
       <c r="K16" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4693507740882824</v>
       </c>
       <c r="L16" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4815210165364127</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4708505865312823</v>
       </c>
       <c r="N16" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.48598362130542</v>
       </c>
       <c r="O16" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.4611000462617064</v>
       </c>
       <c r="P16" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4818681728836816</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.4865880775801012</v>
       </c>
       <c r="R16" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4911303544680503</v>
       </c>
       <c r="S16" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.5038321571659101</v>
       </c>
       <c r="T16" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4871712272930142</v>
       </c>
       <c r="U16" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.4995798463274351</v>
       </c>
       <c r="V16" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4971353275793846</v>
       </c>
     </row>
     <row r="17">
@@ -6247,67 +6247,67 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.470452888438528</v>
+        <v>0.4709725437712467</v>
       </c>
       <c r="C17" t="n">
-        <v>0.4830880060177857</v>
+        <v>0.4728245190675379</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4727235135626869</v>
+        <v>0.4737269467395356</v>
       </c>
       <c r="E17" t="n">
-        <v>0.499645410718047</v>
+        <v>0.4941094765543679</v>
       </c>
       <c r="F17" t="n">
-        <v>0.4808085515391495</v>
+        <v>0.4961056032454816</v>
       </c>
       <c r="G17" t="n">
-        <v>0.4953904855767604</v>
+        <v>0.4899619750100624</v>
       </c>
       <c r="H17" t="n">
-        <v>0.511631189803649</v>
+        <v>0.503096947279107</v>
       </c>
       <c r="I17" t="n">
-        <v>0.4936026199694747</v>
+        <v>0.4991374677464053</v>
       </c>
       <c r="J17" t="n">
-        <v>0.5081064774301788</v>
+        <v>0.5021196199061189</v>
       </c>
       <c r="K17" t="n">
-        <v>0.4637027508964842</v>
+        <v>0.4702300660762643</v>
       </c>
       <c r="L17" t="n">
-        <v>0.4689346058251911</v>
+        <v>0.4774609856149423</v>
       </c>
       <c r="M17" t="n">
-        <v>0.4685572580048092</v>
+        <v>0.4721779350677842</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4853014882948868</v>
+        <v>0.4847954299882681</v>
       </c>
       <c r="O17" t="n">
-        <v>0.4659106444388175</v>
+        <v>0.459747957249802</v>
       </c>
       <c r="P17" t="n">
-        <v>0.483333743514206</v>
+        <v>0.4858447523210159</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.4835983401747622</v>
+        <v>0.480102278977989</v>
       </c>
       <c r="R17" t="n">
-        <v>0.4894300050449246</v>
+        <v>0.4964647959682091</v>
       </c>
       <c r="S17" t="n">
-        <v>0.5060657190831327</v>
+        <v>0.503634671124324</v>
       </c>
       <c r="T17" t="n">
-        <v>0.4808132745541029</v>
+        <v>0.4746288967046488</v>
       </c>
       <c r="U17" t="n">
-        <v>0.5001093368982007</v>
+        <v>0.5063099805768435</v>
       </c>
       <c r="V17" t="n">
-        <v>0.4977729256639644</v>
+        <v>0.4995212915763057</v>
       </c>
     </row>
   </sheetData>
@@ -6464,107 +6464,107 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c5039a397d4ff88b1e66469cc1765bf992bfd0097c506724df6bb8970635fecc</t>
+          <t>ccc818b0c800a05cef21237cb3c4bf8fed151fe1dd60a34d545328371f091898</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>eb0cb9f29a852ee094568ecf83f76859b65b280c6f2f0a67423c0f47cde4d02e</t>
+          <t>a2e9c93c93fc8301ef75924386f30018419313920858f570f89bd6d308f2c673</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>431098a667c082e2bce82a3f5dfd5912d20d56c2c28e9a088a63f8d29371c0bf</t>
+          <t>9ac3a0c758cdf0a6e857fbc8e586d75360659179816b46ce862e5f802db93d75</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>a9dc67d82e9b8431bcac150de82918381e548648c7e9d98906d79f603575cbc4</t>
+          <t>6465dd70c1f8c9ce4a68ee65831036c0c2e6146efe8ac21d03779c915e1bd8cc</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>d462f3fc66f5ff3657652fa3ef2ded70c9c267b84312eb414136042a4f0b4cfd</t>
+          <t>6a2a1882dabb70b562d0835c3e35d412078edae33493b6f893a463068b1e7db7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>01ffce22bcb297423707f53fc3c03d84255799f3b9544d81487025d612fc2585</t>
+          <t>85ca64627469551ff37ee071ea6f658e12146faf0d05fc71f207a4707c6552d1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>f0393305909f8a720616342a76f883fee410ffc8836fb9dfe8c45a0ef937c1f2</t>
+          <t>f5c7825bdea93686c9960958fb0abfb62048520240e5760418d64eab92ae1d23</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>a7e9e58810badc4c0a8eb882f1091eb791baff2f4d028772e1990d077f1c437c</t>
+          <t>0985574bf841f94ebb37f589dae843f16eaf59f703ba45cfb25b8c53f1f30cb8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27925fac10daef2f3b8f7ace703664d3bbfc8639cdfab5851b4689740f05f0bc</t>
+          <t>cc53b6a211f9e7d6c0f6efec622aed364207ca217629e2e0e59969c4ce26f9c9</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>c4421853882e7b591310cd427a70849efc71018036bc467219f356ccd704bacb</t>
+          <t>aa3833c6c48abaf38149287b98cf3d6d5c8458beeccbb85972369558088359df</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>a462ee357a29c55105650dacdee70210913a09b62efe0290bdda558f845fabd9</t>
+          <t>f9c0fc86f237589cc6fbd417248b1cafaaa5fde69655ec29b15c7e6b72bc9835</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>b10fd5b4f2995da18f8d68c23b52f9b2a1fe890b6c321e4af340a427fb5d4bbb</t>
+          <t>6ac3025e9747048a79a98ed8d41f39e57349e56908bb746ab2a9388f58821adf</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>e57b22a2329194acf07148ebcceceee7bb4e447359b5ade31d507dd346819844</t>
+          <t>96814adc02ae3755b003fed49bd0f07d940c7466f381412d4b1641dd86f15a31</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>02cf5ec319f1d224af16a79e31690ab95fddd485770957b712b535bad5bf83e6</t>
+          <t>29cff13acb1006b9d7913debe024203199e344ac299f1e162c87dc519f22f921</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>651f5b62e374968ffccfc9b246fa664870fc52a5e43494c08e3c63dd8e584db9</t>
+          <t>76f0af43c83b65b84b66589148bc897e835f09c70d17bf0ee8a11919a49c69ef</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>503dee552060fcd4b19fe02b2c7a18580310984ec994fc7a6991616da9d1e7ad</t>
+          <t>1345f9b14c15f3f6fca3138712ef4334d728e8c142a39a13e3096556a4e6173d</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>507c99515b6d006cb128a6c2a91497e3c24ce2757ffcc83bd514e0dd7201cc90</t>
+          <t>9afde8036fb289ff9536e6b8833051c863c29b8198d7ebdb76b9162545ec17b5</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>8141c9e981b5d61c785f3ef5aa9ce96316965e10f7c7b846eed85f067c93710e</t>
+          <t>37ffc83e05874425d1ac7873857c1ce3c64bf8758bb9b701b5254fa7be67cbc2</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>15f2d31f9cc3000e5a53d050cd2657c284065b6de517e7bc02fac9236a04bd2d</t>
+          <t>4171a7964e41796fb60e2badf90e1c3e212e1d26ec620582224d476f275868a4</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>fee72a52047ad9c17309cb965b09d017b6f010b5fea4ecd1c6e5b5971d06554f</t>
+          <t>1a2d4acb3fa696ffdf9d3fbdbb3d19339521e52259cba585966b24d02eb0848d</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>dd3c64c9d9fead77329dbf5f4e40efa88a7456f3fff55d68536b1c241adfe01d</t>
+          <t>3b848ac9234b86bc1150a7acab9236bcd7a1d3b8d6115e7824bd8f0947b44863</t>
         </is>
       </c>
     </row>
@@ -6576,107 +6576,107 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>d256f81aab882c1c7f16ea101424cbf8c80d5cea49efcab6893f4a676c04ee3b</t>
+          <t>181162ecbab1bf244567276c14e9270fed73a089291e2e1c1292552c185dbe79</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ac53d055b4f75ddd8142372c3ae1ca5f6e55e9658840da3f971e61bd06797199</t>
+          <t>fac7dff035871e017a26c920568f0e107c16dace64345caf3f6bc9bf8bca7768</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8292b03354834b8530aa18d3cd5892a9e9b6870c1447cbfed6cd5023f0d8041f</t>
+          <t>5038be7595ed0b497b93bfe4f5c15abe8482a5638b34a5fea524a7cc6e6954bd</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>f1d70992606c753e1038eed6ae743369bcffed6d721daffdce1f6c0f354fd4dd</t>
+          <t>57b9ae0b19df9cb9daf40442ea24e7be4639bbecadc4231a7a0a67a63ceb9afb</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>96a91f453d3d014edf8688db08c86197f887e292d6ddb49957fb9899d5c3a151</t>
+          <t>4d70f24c2da8f87299e06413a302e03fdd16c0c0dbd8bc2cfeeeb55c2f3d506d</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6056235ee1d3c0ff274e4138542640120de5ae45a0987cb35f25e1d77a24af3a</t>
+          <t>ead4dccbaa9c036de2ab70ca3c19fa4f970814a98bef2ea5a0f27a7887c92318</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>5beb20bc406add59d8b49eb7e5d24206fc18a630be59ca8083d3024c1a9d4b42</t>
+          <t>34eadc2fdec9f74c3e025cb8a01ceedb3e98e5a36cfb198c8a21739531344afc</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>45a4c7b14eed1767ddbf13a48e9e72c4dfe424536e13dc7f98b14eaede4504ad</t>
+          <t>7f12578ba760c654ed8d368ca62d6070bb9ca1ce3c1ef8c21a8306f196e6c9b3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>45eea618134eb622ec523f8574c72862d4af168c4651fe7b5951a5c465c81534</t>
+          <t>57b4c97ac53b2924d807e37a0dc2df89afd374d4a2745ba88e3b1b0722e804a5</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>43f4507a3633208f23e5c4e7612e2bfaf88b101a920dd7bf23d6b0bc484abd9e</t>
+          <t>741f70b13ad81285730150b0e771292cd01ffd175986ed239350c210eccd7b85</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>b5e2578b4531710568dc59bc7ac989623989a3fdb8dc96e9e0cb4de0a21a1070</t>
+          <t>1752477240ae5c52444caea60c1bd3cbd30d108a15507df304aab98c3176137d</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>ff4c9ff9c21326c3d7a00e5ae477ee390ebb9dd6eaa0b5ba14dabdac1a3df2dd</t>
+          <t>6dd75d614fc254ee6d4a08e4c1f044ccd8c4b13eb28b961f072e0354f6c4cee4</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>f3c2327427a8323e46928f874b1e5a2a43447be15c0758b71b3cf60fa4a4edad</t>
+          <t>073e8a7d749bfa08da6e87508e05121326742d632617bf1e5ad82a590ca33952</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>68d66fff82a300e0280bc792990b8314b0220216b86178c53926a2b19a21b63e</t>
+          <t>a1e02007a672d5d05c6e697e3036d11c25fd59ee65c65f7508beac8303343030</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>790f24bc71165599c0f0c2e86b5d5a7ce5e0d22165fc8e7b7189dcbc9ad7ec6b</t>
+          <t>092e06d0d616e0e2775dbfc54b0ca1e7245dd8aa5591932d3af3ebb8f17fd8c2</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ee6d1b5f271a4fa0d969f26c8e1837c556dc436ab871fccfc5afe6fca7e5304c</t>
+          <t>1925889ffcefd4cb86302b57a3abf85cb47238af97906cd7442990a8207957ce</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>38e6a68a8f6226c71fbd11571c2dd5246f414b8d799f731fc6f741507f7e0e16</t>
+          <t>6755214f6b27cf4ecaa37535005230eb0a7fd8fd1e344401c8c72ffd033b7832</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>d26404d29a157b4504bd15196923bfd2bd284d048543c483668367b6874432fc</t>
+          <t>e0cd1d220a2860e1f9553a975375d21b2bcecbaffd33e7b8fb8be98c0b74070d</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>18a0528c9bd192744d95f291b0ad44d0a552d3448d150f27974868eeadf74dc2</t>
+          <t>86ffcaf94268b222d57b0e2f01ce3132edba21f55229954f2a5442329050c15c</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>63789633c7a13dfd909deb4aaf1b2444f29cf16b18ead443ada41076c40e8e4d</t>
+          <t>729db2730cb2f0b847eb7562ec4b681a5e3b06ea49dc9c486b3ad41c526be7dc</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>3d2fafa4443eea6a4d0fc4f97c8286ba53630c6989af6c597a16022ed5b68bfe</t>
+          <t>abbae29ee6a9b1c4c2788a9dc0cee968babf33b2b0ac3555d4dc0abe3c3ad837</t>
         </is>
       </c>
     </row>
@@ -6688,107 +6688,107 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>42e61231775acf31bc41ca26b20a077a46c94ad44a177a3dd50b5a7d0c2b0b19</t>
+          <t>126f3bb20cd495eccab56e0d9548a0c4cde5d25fe1eef7f6a0797009aee81b71</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>08e05b9e039ba8dfa7bcaef4ab2c84f3ec037ea8ae1290bca3c00f6e4e8bfd32</t>
+          <t>76fca2788f89ae9c2cd3bdc6d992d6f4cedc403178ad61c5c6fc342264469f4d</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>f1b30ef75d9fbb9c0002ef3783f6c2094723dbe060ccd966a7cfaa73319d1970</t>
+          <t>19693c1d4b3dff296d4bd4b96a7e22233cd6675486064e9483ba042dd8e89d82</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9c79848a25252cb86ca8dc133f3bb5f86cff62ae848c70742bd863884cdca571</t>
+          <t>9ab79b3c77ec817eab16ad9d848fa282e14902ef94873e4b8743ffa692a3575c</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ce8c96141e62692e915fbc9199c34c33a7b67421b86d759a0625960220e3131a</t>
+          <t>97a595a029dc4c1dd9dfcfbb146d9fedb0e9a4da3bfc5955ed07840b1edff188</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>c115178352d4489ae1a58fdf289c1cfc86356bffdf8306e3479bd423adf120be</t>
+          <t>4c9ffbf0b7ec4056c6cfd846935712ffe99a41eac534b32d6a29ba18305e4a41</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>b2586c17fa5abaf5bf0d7c185eb3162168c56ed778140bd1ad59a05762ff6c59</t>
+          <t>dcc7d4c1b5186800ea210556f63bf63ddf87fe7e72ce496c18cadfb02bc036de</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>64a884eea786eec088e533176b40f81726fd7c9bdf5cd638884b76807715a765</t>
+          <t>66cd062f21ea36f39f9ff05fc6cec4ba31b1132ea51a0045deb1e440e6613182</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>46445e0570e9098f6efcf4455bc5c93ea14dcde55b6ee620662918bb0a30bee9</t>
+          <t>b85c6639c072e63cc773536516b59bb10d8bcebf174dea6e2c3eb2cb28ce1be3</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4801c5850346353431d200d0ae7a8468e2e095f1fce3f0ef4f60d34a34b34320</t>
+          <t>4708e4675f92cd46dc5098f1f695d6517cef9a515cc403b9c416d18f4bada865</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>832a03ea9ae11c836577715404d0b1ff8bece785fb06885513669bba15aab336</t>
+          <t>1dff3efc930988d43b15108c1f3e8258d5ddfaef8ed585584269e27c11b8abe6</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>9e70ea71c7b2c2dc8793ec6452c32cff63162e37d3209073539740434bac5800</t>
+          <t>1f7765cb87bfb4b0aef4bd081ce7c7251608ee26616b9d295a207a8c98c5e811</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>a7485e6a8261e6b4abdc023ebc7f6260193ec5a3b281db1816bc94f192fa7b62</t>
+          <t>81c01ad934cabaabc4301234dadc7fad7e1562d3f34232faa3785a146ad3dc5f</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>6d070b8c800ae56f3e69571e7c22523e31594615e7c9f661611c51e1d0513215</t>
+          <t>34239e75f4b8e8578f8b5c5c193ca7e38d5b7bc5fc1ec84233d1f160e1e581be</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0461e1c87f85e76f41adb72052615460f10c89325d36f4298bc9288f55d97ea7</t>
+          <t>573f38f173f5151fa9fe70bf2bd4e4f45fce1d4b457bec6cdd4a6be3510e3f8e</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>a4f14b41674ccafe594ae8efcf55b126145b3488b20e974c97ddb23c5f0827f6</t>
+          <t>ad33b3e33956fbe0ebce8e14e95fcf4bb303e3f1e71961b9b6348af837dd8b26</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>732a1337bd416a152f97b4a1428486ea88d385b95fb95776fda98039676099ef</t>
+          <t>5088edca6169ab779dce344bec86269e150c5254e1bdf2cdebf3ce5a5a9e83b7</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>f31e2c75594224f05f0245feb606913252a92b372f04e750529ceb5e90c9dec8</t>
+          <t>a920d5d8fac999b1706fe889d1fe688700837a3e3ba1d4abb7e9ce2cca41733e</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>97f7a3b5bab2ba70f973ae68022a339445aa16de0649bd0a2354c2a58527feac</t>
+          <t>4c780ec8769b309619064ffd4cee0af085f85cbb4c12d48dfebbf271f7e7a50e</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>a7ba078fcb69a401fd4c208cc61e79fc4dbd4e891cac517a33dbcac620a7e962</t>
+          <t>b3e0f2fba33d191973f2f2b7f018ab27fbf7601b3b9904efdc37aeb3bf583e00</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>d3370b6ee41e5b8f9479285835b89a3c0f38eb927a79c49a337dcfa1a85e2028</t>
+          <t>3783ccb6062acff4e2e06dea1d6aa286e35f9bf35215ec4bc07cd25d1dbd9900</t>
         </is>
       </c>
     </row>
@@ -6800,107 +6800,107 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>61170ec8016971a1ecd743699f3d932a2840edcc0be005f88633ca932c5ecf10</t>
+          <t>2c463b45e110b554e9802205e092ecf804134e2efa97bded9c765b74e7ca3a44</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>d9178702bae116bbd60158aacc9b9c56907c8014650c48b06631c525be8b313f</t>
+          <t>f767f0aa9f3492118917247a7dae523fccd9ec6d44f7990332cc65d4c566b46c</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>b9544b5174d8bf1f84d5bb805942fbacb3bcc382f48d907b60071d4d4efef71b</t>
+          <t>c59929772a5b04f204c7562a5923c3c252fd52c6b2ff28989cdfe53bd4691923</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>71fb8ccc52edcc06722db680315a9a304781e5d7d58c18abb5485132ca53177c</t>
+          <t>867c70a0b3e70f0bb20d3ae88999e79de69ec2d8c50886ea7258cb51edd25042</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ae62603984caf68fdb35130ac57185386cc8eaefc1204c88f40849003cd12452</t>
+          <t>aef684ff8a2456a99eb8a7325c7862c34d6e3538b39c5ba1102b1537b9d991bc</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1c1cfb2ab6d53d4c135df4515485935cd5ba90d584179c0d585e4e9e5cdee586</t>
+          <t>713dfff9dda425b8dd377a2c1eedebd4773e5aebdeb36f4cecdcf7e372a40f8e</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>82c4e02de69f6ea36f0050d267465c2516488fdc2f82fc8be7e37e9210711134</t>
+          <t>2bb93f76aadb28801a5a94abd4fede43a97b0336d8da7eadd9e994902a53d0cb</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>815424ef4c421c4b1286a60a459241a866da77acbaa3921e9ab1d5fa5965afd0</t>
+          <t>6fa62fce0f718e57ad55e02bd2f4ead312f711840006f535ebde37a7d91b39e8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>90e6e2a25870a712bd11e90c09f6c738ff1a367ba8fd9999ff932d9b9e6594ee</t>
+          <t>b908159b6603c8e58eb68ff2cd09523589bf9d4b6df5bf62c3b78dfe25c38960</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>8afc722c7c8a1fb7266405c33b22fe379edfa5980eb93658e45eb054a0ebb8b3</t>
+          <t>ccf036be5027d7f057a44747af9f0d0531ec23b5393cfc46b3f4545dd418b60a</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>729c809585de42767c32d4f0f0c976c8f6cb67198f27e8071ba5124834534f56</t>
+          <t>37977287fa5535a7d342f4427e2713459f17035fae027193a3d51ca00e22eba0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>ae13ef2835558f8696403c80b38ce766833e98e0662012c898ce1aa651512dd1</t>
+          <t>fa642cca0cf5356e6c7c94b74a669c8ec30f8e754a301bc39401165ef6948fb6</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>6d7fbc3e500a3924bbd43694a6090efef20a632bc2634be857909d77b9c661cb</t>
+          <t>58371be6bc62c1fc6edbe5ca8d370f5b6874652aa4a6a848e79c8fb110f853e3</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>59820e8fcb7909c315c67a5e506c30b135067e8a668dfd5ae2e3fabaaa7d6411</t>
+          <t>b98e47a09894c4304886b665982b76fd230b1370ee72b04ed588871509d3ee84</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>a9e9f5234f2b57a2e72a55e7f213af09bc3bddcf2565321cc4a0e6f96897e2d3</t>
+          <t>3742909408dcb03cd98b3da3417ed9c58e0ff448aab7d432d4eeebca3e336528</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>aaef75ca375acccd0fd43026a3e651e33bc7b7923b118f44be9910255d7beb43</t>
+          <t>e35e140f809fa2155c3ae826734b03c4a1842aaa51f2be9791f861dd0d77b1f5</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>d79484db429b6fb3fcbd0fdd5762d81918a73369ccb49e3884542316cebc9346</t>
+          <t>71807fee1c3030a5b06fde696a05ac18bc442c37202572e1653e46094f084454</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>d13fff4009c5cc242af36754b5ea6cb8e415a2c6a28ef9e285637c437e9b349b</t>
+          <t>ffad98a8f597de657a9f86be5058016bcd3db10bc9da8cb304475ab2b8638ea9</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>f51562399c5a88b95027c9ca1e42b7fa24d9a242ddacd0ba7494b7d77471c07d</t>
+          <t>f4f4fc17859e94dd3c1aab3420aa1b532b9fbd95d636ce21923ad3071256bc25</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>b7f060b4ae6cdd3f5fda72e18534d3404342287d65fc84eba9b66e34e804a6d4</t>
+          <t>1029fc9c277ef801f29e8bd8e81346737bea9dc61c64ba06336c481cefc7643d</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>5273fa34080f24666534e1e746a3c0d645cdfe028de463ef8b8545237f94210f</t>
+          <t>5b1385664c46f22bf4c74ab80f94b1093c76e6df61013fd502c3f59bb6c9807a</t>
         </is>
       </c>
     </row>
@@ -6912,107 +6912,107 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>c50060680e7f12e80e5dcc2002370e9e3bdefbfa1aa4165e2d85121769270f41</t>
+          <t>88e3adb713fa6eb7c482b4507cac7eee7e58bc6d067f0cb7c65f5d16e182b534</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0456fc55eea5d7a6779930dccf1a45b7fe40cc22727838877b21a4b4deb01c2d</t>
+          <t>229e7ade4147eec81679c5346f1c28c715a478cfad1b07db96094c42e9f6ba31</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>309dc91f03c910b1a79c8b893923b9015c14a986f90a0a55c1d3dfd8482f7466</t>
+          <t>b6a575a9eb8141836be58ab8b5fce26f5493f3c8c669774ab0a92c475c08cbaf</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>18e28f8884c05737350e1410f1be7ed2abf0d5349f7c92d62918c2a5089bfe5b</t>
+          <t>6d3947bb82596d8763d11be0f0809f4a180f3e02ec5111fa36a8236cc1a7743f</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>25ac0d99bd5a2f2a28544f79a37cbb7f3e2f03b5b29fee7d68d0f5d669a79740</t>
+          <t>370a44c6fa0d38f08f7ab6167042e408f023b037b36d385801a5508250e51f37</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>33250d8076d691993ba61d4a854ee7f2d5b5325811410de95c390336b5206ddc</t>
+          <t>351751250ddc6e8bed8e180b2c22877d8beb12ba547fba2d19627b699658333c</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>819f29c9e86495a72df05cc4c3e4be70354f14c1f05f70c9fa5b6a178823fa62</t>
+          <t>f6f030f8a14a1b452927e925e22cb19add034a8923379385e0653561fa0a7a1e</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0f11ee258f63fc1f5c2276c8cecf52ed891413ed08a3d555c5fbe2e293ea604d</t>
+          <t>a991dbe938e6403fe697ce2c73604e818cc8530e31decb8a26e9d937f9892672</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>c70c7ab6c73c6d9ae8040b80177bfdf35457bb0ccc46b2b7efc6434079b87fac</t>
+          <t>7a738ad5db98696009ced9cea086362176f28c644b0daebab915c72201fc5bc2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>e87a4f2d5771883e8ef91894784ec502356c4405868b05333df10034626e6e4c</t>
+          <t>927615f810fddfadac76b9942554b83d4739967cd09c8dcc752506692e8a3b33</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>4ee8a4386f5c7ea6547d429618e3e97afdc1b0006c764ed67dab8bcd120e48f0</t>
+          <t>cd74bda730e2b6c808c9e64dc15d7e409d02384efb08f61cdd6b032649fa89d9</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>16d931894b2fb98aa15b803621d44f1e3d1af77c55e435f8d33fe289430d58ea</t>
+          <t>bf409da4b7ab6751b437c5f15312612eb83ede58a07cb2ae8ef79ba99572385a</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>af84c35e4b0fc1a7b61054644affbb8b5a4c56e107ed450314404ad5e92ef1d6</t>
+          <t>1912be1602faaa241551d6392fac5088b465204c65dc2158bc48acbcbd58db8e</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>ccf3174b6f94988c34c35df32a0a192e8ff79cfb59c99731ffadc203a35d0185</t>
+          <t>27a3e01c42be8dc27ae11d9f73400f64e223d4fdeb0c510b1d23af5e71315079</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>6f9552e460e4bded54d6e7eaceea5fc98564df8c7c993ada1b944f5fd210da40</t>
+          <t>691cb8fd50e00de2d169e56b559e17b2e86db07dcda99235e4801ec6678eb943</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>7c732a904163c9b564336ae8a4ae4b0c63598e8f2ebd50ee4554367a69c469c5</t>
+          <t>823474db174a91f3e5667c44dcce2e0bfe5d4a6b9f8c76b32d80cb1c535c39e9</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>11d1b05f2f15730744b57c69c66f568f01e3f7a888ace22c932dca5ef02a1433</t>
+          <t>d4ceeaa329d194c88194b758492b617d5e3678265338c576602f4ac729479240</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>573320f4eda637d4c997f7882f0cc3c1462a304d1047b5369d8435588de2f42e</t>
+          <t>f9ae674c2b8baf5503cedcdbf9c9aafe0883bae9fcf887416e24df30b22a99c3</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>7b53fe1abbaa3d9d5ffeea7312d6cecdbc31d647acf67d65cf406d129f58b7c6</t>
+          <t>178c92a224f3b32f1cea152fa496a94a63905b69e3f593d49e9cc4e8209e07bd</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>27c2557c59fb0b8ac78bf2baff28f3f6d6a4a1a295ec3b62005d39b9eebdd3f9</t>
+          <t>37e55da69c8a7914d80a3e6a8656ab888d333f0d7344667d638cfa659fae6714</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>347524165c676f55e3c3a7067de787d09a938f5874d3be0a2235291211ab115e</t>
+          <t>4e3da12403773abffde65421337f66980b417c8e156c0c0d03ceab6fa39b327a</t>
         </is>
       </c>
     </row>
@@ -7024,107 +7024,107 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9e4b04a6e3fc6efadc1afe420a2b703db1775d2acd21f8a52c19eeb31136da32</t>
+          <t>de04ae08db95aa83373d0d5f4ee3591b211f2bf89169aea76b1bb6d3af8b258e</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>fd091e920f3823b90e8b06dc2dd1492b33215540a09055005d713072d75ea9f9</t>
+          <t>8dd260bb52897c64610953255f7d35876fb6cbbc0e3e384877b57471e4cdd5f6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>20e2a1850483f76f381e27a9147e4125c58b2c6965627fecd6ab8a0298ad495d</t>
+          <t>d2b6476e6052a993427b636bcf5826b335cb5c73dd633d136af7630b9ccb8318</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0d052614eeb1134c84d6f23d3818db532bc80f4e8212ed0b01913bda3e43de62</t>
+          <t>c0e59b3bd8d0d8ec18aec0eb08cef37a0a90e02e251896156fb019e99f357c8c</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7c42221648ae0b16da585fbb7795a36661e85bc17c037350fced8f9e157d219f</t>
+          <t>3244655cbf1b267f97b5b91423a1e391e8524b0c86b25db04c8fa4f35033ccf3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4549fd4e000e9977294f8e351931638be9f9b2c250815c09db5afd984e2aee92</t>
+          <t>8559f1c4e6045d14f4313cbc45c173124a1073db492d00a6b7d2162922e4ee5e</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>e52620f9b27f64488f9f0aaff93ace74e2d018d9861271350478092ab0e3abdb</t>
+          <t>de9371cba1bf4efb07890dc0587fe75f86308c3f779f788c4bfe5952ddbad53d</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>7a3cfc9fea183f8fef950c92e5acada8a4804d3e88e15be18ef87b06b59095b4</t>
+          <t>6eb1e5f1554ca49221466a2e498c971d7830d04d3888f64148198fe3515fbc84</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>f93d54c2edfd857fb28d999bd385a6826d6220127a11f975e16b68902dcff2d7</t>
+          <t>8f97e49216efdc6281c527558a9a19f572078aeec26318cea649bed75014d8bc</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>6cc4fa70562a7911bf1b69a076a2de02726399e85dba3daad4b6ffae57371b28</t>
+          <t>f2189780f0cb375124a41275aea6718fc109fbc0bc248213a23367d1d6b9973a</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>b13e817a4c6e5423a56fcbb8e29aef3b0a5213f4d95ce7634cb23bb195858e62</t>
+          <t>74daf38ba7195a588417d99d63f66d2745198b8983a8f2f3736a2f7aa40ab55a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>f7d1721ee5c19db9f7d8f032ec889e528ff599a3626f402c97c847163c5a2cee</t>
+          <t>f439c519c893df4631539dd8b88845712a22053b7e18bf2248ee84fab0fe2abb</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2f9236dc5add086a4523c369be9d4a8e50764b3bd9d2be3065629bbfd0c3ad23</t>
+          <t>1c466ed32f0ff78606d6c15a67adea10d45514f6feaa256b1628e8dbe2bfd850</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>aaa3cddcd5d5d919167db39f6edccb3e3ad46048ba2518c2b0e5a40a9c68f4cf</t>
+          <t>20fe8c084fef5b1ca4f266a9bbd64bf166b640e8168a80a810d808060e85a80e</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>6cc660468887bf1e6e588e372c763ccbf6414145cb2a3b0e2ca25bcc6d50b087</t>
+          <t>6710fa44a278f37df95696349ffea9fc108cb62b71d8d4a0187cbe08f8572f41</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ef1c6acd221792500d7f1d7b276e9bf8a01a168cd3e4fc87fb111e0d961712bc</t>
+          <t>dd4a561cd97f4c397a03aa7cf150c54eb5d04a7de4a0fa9ab9e23927f22993a5</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>9b26afc2c65050baad0b497bb6a0b8ee6f4e0f08ff15710341709f562d3a580c</t>
+          <t>06ec43839dcdc3980b51929a0f2e8eb0486ac3af748a0069d7469487ee09527f</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>9c11af4650ab63c318101a9f2dd856b55fe137e57cd788364d535a1ac64c1465</t>
+          <t>75596f0507b43d35e40e1227ebf2a264bffa91c1498c9758ae171a901fb369b6</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>65ce4a2bd411fd931c04a28bc01bd46bded9c09c0a5a5df52cd8286a7daee9bc</t>
+          <t>a21184abdb9c466d24258840133ecea392389cebfc110c46da16f66d6ccb1aee</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>fdf61999641271685db43ba0daf9b3dca24c8c91f485c3306dfa0e3139ca0d13</t>
+          <t>08bbdc79992720a8694a9f494ced8c852b08e5545ce01da4840e0c2b848f8b7f</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>7c8f280be09a3e00981230e2c891ed04c25ae71d47355bf984370f525975db1a</t>
+          <t>9d26658e3ee079c2a2eb7c495b8a8b35402e33140700fdf61e2c560385c2357b</t>
         </is>
       </c>
     </row>
@@ -7136,107 +7136,107 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>14c173a509ebe1fa801e15d6c05b102f72fed47e135a5085706a817b52b86854</t>
+          <t>1e4527b7067fd25a1fcdc6a0ad7e19db624f7747067abe19f3e03f04ebce0e3c</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>046aee8f8ca363d1e89be5a467f057c3d24b02ccad71479cbee865220c73c585</t>
+          <t>f6f57cbd80e8a71565ba7b9952604881cb6783293ba51cde365d1ab7372c4bc2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3b8f5fc11780afc061c8a46e53c2b03030aa62db4cd4251df6a091682a3a57e4</t>
+          <t>95e1eda8263ebcf36c476718330c155385fa87daedf1c20dc3bfe6228a5c4204</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>38da49749d10c53dc87d9ac3d30d7b874ef18c747169e0dbe9c6551ccd9a1854</t>
+          <t>22b744f55d21c55fc95679949f0393910e71d82d31e356a0afd28881757fb146</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>aefaff15a446a5160a87cf52dd262cd95e036cf08ca4df53164e82b036c074d9</t>
+          <t>089ced5bca4153b23d07ef2f673e5b5250afb429dfc5429e4c747182f964833f</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>a4b03c0fd9299361c29e46b2e8c34bd4c2f7087fd057c7c58f4d932a156fe900</t>
+          <t>f51c98fb460f76e032fac817a752105414b6ad465ec1a6b570578f1b3f7687f4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>764c5e8288ed73f9b853dc2e057bec55d93ef4f9cf52c08cc8050e3c69912bd2</t>
+          <t>950e98103f9eb12c27889e580934f6a431fb3b6e13dbc8e04e49455b31e706d1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>c581468654b7e82f59baa7cf01720a8fd23ae65cdf86278e275fd7f5bebbd758</t>
+          <t>d6f0f023aafa58c7093bfc717c207d6632ff783c9491d513592bd0f5cf86d7bc</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>d836b39c1a2555e4bfcc074858bf6dd4a1c40896be148f853ac62820224c0a4f</t>
+          <t>713c770fd9bcf3ab40cb634edaaeb2a6ab0137307ced33476b8c3f6b796036ce</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2ea9bfbb1db8a1da864a68fde507f5340c256479b9789c0d932afc8770bb4ab2</t>
+          <t>1ee1fe71e68cd24299321d0aa87cc460e453dae856c10b6fecbcb7afcd14146b</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>8c8e7cc9412ba732c01eb31db3e6a5045163471c7b8bb7508738cf97618e76d3</t>
+          <t>0a7cf29d79c781cc5ecf049ef211dc77c3e561984d1ddddae185b0ed8ebefbd8</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>8da655965535fbf90f798d8eb72e237a44f6d0fab8b0228c0dcfc1116b615f63</t>
+          <t>e299a40c50eb1eb18c53dd3205d72a39cb446c519a280565c95a8695dd4b6a7f</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>537ba419597bfd31465c6c22c5df258fb11ba435c20e9297fa9f7d0e5a069d75</t>
+          <t>43085103218823ca53faeb9ced98c4649b8f5f825e2b32de975254a915fb0f19</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>570453dad37bb8f2d04b91423fcfefd373778f3ea73ce65ff0bca8553ae5dead</t>
+          <t>a34852d251df337c7accebbd77bd3440c103b490bde5fcebe8e7578010b0998d</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>fea304dc7e63becac83d4c4ca9b7d59be7976980ddbf628c9d48c8ed40a6a1ef</t>
+          <t>82b804f543e4636940ec2caeed412c9aaab6deb97d137e3f76f0f0d6d2a0b6b5</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1124f8f765f9a197e3b9ba25144c6bc43441ca4fba9ff6d6ee05fff7ac85fee2</t>
+          <t>90ebf5d1f2dd7265c8b6b6e94d69aad84dcb6f2d888f8e41080fed3014f22d99</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>fe736da57e674200d5905775ad2954ac05dace1f31808a6ab728d3eea3e360d6</t>
+          <t>eed2fd03611dd622114b4feb6f906b09e8f43db924d43029098083c6b255dc2b</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>6429519f31723694f5d74e894ce5324a75c9ab5f28f432b61f665d023f6b8720</t>
+          <t>879cde4ae0d1588b9481b74e55d1fad1015831757c139072ef224513c4ebee96</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>713c7fa8a0fd736bc99f6b865c2775a5699c80aee4224fd6cc80087bec110d04</t>
+          <t>b0475fdf65d287b03d1ca7d243d7a0141ec7750c47afa021f9fe308bc899770e</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>e1e4d0ac994019d87cb30d0bc0f87d7265cad216475405237ebb3b4789952d7a</t>
+          <t>f96babb03f8d809e7c02eff255018892f9a7ce93c0a4bdbfb9c1411b942fb100</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>eeeb3fe3e11504640bbeaf8dad612f50d53f502cf92c062006c3d2b271ef25bd</t>
+          <t>c144fb3f4cc4a5b6671f2ab2ec507cc8b2bb8b03134f7b74011f914a6be1031f</t>
         </is>
       </c>
     </row>
@@ -7248,107 +7248,107 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>64e56d7a2e5246cab7fe4182d88e5d3d6825f9023162d8fe6ca634d0dc4fba47</t>
+          <t>326ed71dfc967ffff9356c3e152b22afff980ede4fa94b45adbf6a2bee852361</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>e465d9a0e441cf02b26e47165c7a69bd7fb8e7a5e26cf7cab630edb2076d187a</t>
+          <t>c0f8a9363067998a0111cfbda956353989b1d9fb489f7049fcbdbd50d20ff33b</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>b52d2010196a076e33e3e53ea75133b32c21338a3e0f72f184cc869ffcad3a3f</t>
+          <t>8804791b1d8174f92764508b5969f314cce115556a409302e48969eed049edb0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>f33a70bb95fdf8a404846dfc34f6acd7c4d791df9498078b8955805c8fc57424</t>
+          <t>3f916f99642e508b212f25c1310f8233921694eebc18aa7cf6d63ada4c56d445</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>551d0a44bff3758ff2f19471ac1b1dd59d223a3a5b9025c20c8ddf5e30f97944</t>
+          <t>cf7b62a6560fd841f13d927d0e72aab01388625d35837b889952c53bcac7a08d</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>8f9a442c1f3cef32b378aee7b128fd45ecf509c77696045653ab918912bbb0a1</t>
+          <t>e1f3a419b5e99caa0240fbfbc7ec5365aaf5b93c81e80b4919faee66a6ea045d</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>c9f3d7afc1ddbf01e6bbf17d77f776bf0ecdfbe65a940248c3f48908d2e2e216</t>
+          <t>b7849d03625b6ca2c016bbb617ed08b0a60824be398099028190f68d1ed46b09</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>f5584255c323a783c490a923bd162fd239965b0b6dbeb55a50d69d442342dfa7</t>
+          <t>b94160c718c6949b05f1125cab8560313efdf1bf265248a02b7eaa8c4a0c9ce2</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>62b677a0af0dcb692fe8321a7cb4b4f8e9eb5133408efd6054f98c98bf435c1b</t>
+          <t>6fda280b10b2335b3422a3fc58815402c8aaaaddc4eab568845da883012fca23</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>64c459fafbe6b16cfa07f26d040a4a92a54d2dc1843e5012962cc8e6fc091182</t>
+          <t>1d60b8dae5c824cf367655a27c081a21f3e7e224ee0fc3b0ed020d44d8456e43</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>b1186ad6aecf885ee732821cb075f5ee4712b9619e603236ee792cf73b5ebd6e</t>
+          <t>4aa54e1c86add1a957a7e92e4da67b6d509ea5f6692f447d6f38b2010936e42a</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>189b472f8493351a75f2fca01219a75796e11d24ed6c85cf9e1d31297b154812</t>
+          <t>65e4aecfff7c8b232dccc2f00b1fcdd30e6ae701599e0399b9d924154f6c7911</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>1814f4a37a60ea16342c580a04b6dbb0b99d4ae98dda802e37577a3108ea636d</t>
+          <t>569df9bd6841c66c9b0f84e96c2b88654173ba60c8672d0fe85eaec6c625bc05</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>656ae5587de55fef575bf12d35d0ecb413fdac35fa01172b20923cbc6933e55c</t>
+          <t>a7b52244e27ffbd88215e82af83fa6e68c7300004712320951d79c76c4cb3cd6</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>a242176bf659d613cba20d53f1b4a71b16f940c81583806c796aae2dd36e0da9</t>
+          <t>5b9b64c626c6f5139cb5ca24582de1176861910ae0996a3725c3c1874c8eef98</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>9da92d773064ac022c743e48a520de52692af46b07a48be961f738db5a1c2ab0</t>
+          <t>efee89d2967c72444fb5f8353b7dade809db3ecdf889ffc3597dc45dd8c14bee</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>795704bc4d836e4fb933f07a97567efb5c025e8239f080c379f8d08f6b33ec0e</t>
+          <t>9a4b12eca0b4e8e760ec7d6706a654c8073a38a35dea84ac9532e5127223a2e2</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>ef5738ff718a96e817c32e352008215e2c11a1b284808c0cdbc953a418c04f35</t>
+          <t>fd14313a80a20a876520c6ffcc7e5ba73c44b2fd9257f8b6b061e0aacad5bf69</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>5be38b89be56355fd98a6a4bee054bc088ae127eb96a7664409787e76b80c977</t>
+          <t>abd1f0d33ae6ad09ac44ea9d5975836345c0eab9677ea268ee6ebfbd1b6e1cec</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>17e9b8021712bc28cfc9891ab99a1b5d137db1b70bbd95b3885d63181ed07a11</t>
+          <t>ea0d93d459fc24286dd4d5eb7d114757bf37923e082c3edd31598871dcb59254</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>ce35c4dfcd7029dcfd746fe9de8246e589aa3be4194de68427fa638ca0316b2c</t>
+          <t>799214998e8a2f604adb5ca1b6bf8689dbffe2cc8102695ba2b0407a93a28432</t>
         </is>
       </c>
     </row>
@@ -7360,107 +7360,107 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>b7ad7574e486d2abb1a8214ba494ed0eb4396c24dad21a5a106e2f57809fdf30</t>
+          <t>f9ee3aadfbaad0491fc4e3e2d72845870e6f1eaab2bb80eaa631519ceec33bad</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>bfb4e51d588d15a2fa2bef2e9fae4b4784e08dcae216115d8e3f9e388657d7bd</t>
+          <t>ebaa468cd55e8df944c3f5a18c380ba8a1eeb62f4c4bbdfab698276e7d4a3261</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0960b7d65a1a636088a9dbdffb2194da1277c4664cf27811377aa9b9dfd907de</t>
+          <t>db088d3cf1b2fe3803b5d29d13e50d6142f7cd63ddc22ad770a7f9f4927a79cb</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>62972c71e224d5759c1684e905bf362f7cda3fd68379fadbd8245d51f805067b</t>
+          <t>8b1f2586b8ab432609b9e5e5f867ee5c52f8c79d1f6d6599dafb2331d08c02c4</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>509886c52d42eeafc9dfb167f56d99bc40df2cb00aa754fea953e24b2a400f28</t>
+          <t>f6e804fbec33192d1660b2d5b4037e65bedb794f637898f5f1aa945db314af5f</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6be3655fa81b2fd0c23fec5a5cb93065766061a3b1dd9c2d66088f6a438c4a80</t>
+          <t>3b48e95b4c5f20f6d772b201bb7aba09a9a720dd6e79c29294cacc102f09d934</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>5cff29efda629b3a6aa8dfa89de60ac152598392fbe6d21eca0367d42c78fcad</t>
+          <t>71e94d94c9dfa43762af6f63ced1d87ebbb5dfbe9fe8db1aee41cf86a4dfdf87</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>01f9ec579a5fd8917b2a29fb66e7e8941b9749d2dbb67b3134c17b64006d8f2a</t>
+          <t>1f2243d63252f77d44ed45c20ac7579d140fbbe044d8f938a4ce21ff347cc382</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3ee2e4495584af83bb09f7322065dace6a185f140ef3a94b6750ab3dd4b700c1</t>
+          <t>5c6a9fb8d4b75f6955dce6bddba712db09835ec6d0589f916cc1f11c2af67e2c</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>80c21814c2519232bc1742d907ea1b2f05c7654199b38f500d7dfe980875d472</t>
+          <t>2d36de953f10ee28587dfea1e56c752117e86e9ef58177080472f66fb47824c9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>7f1a12f850d71c5b1f1d7f0c6d3af48fb75f24b89f17e0e69002e482428e7f96</t>
+          <t>64ec50026c59b037b6366c0d8c69df7d6f0224c2b524c083559418c82f803a1a</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>89d92fa721e69379be44f832dc371dcc884478d6a6b8a45f2055bc8c0aa15f07</t>
+          <t>5f41491e8c977b6e635d9d748a2c1d33e617a087fc0dc7200b616039fd1bb175</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>e4e36c2913c4c7ad0b7560828f0d0e7daa724413a0172efc8da007d8f1bb44db</t>
+          <t>bcd6f4afed35c271565d180042734e576c63b4b73ab8ba246bd2669ef30a3a2a</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>5aea70df53ee0f9a7365678645dd0d0e432d5ec661f1d95a39709671cd37c735</t>
+          <t>8e1c3a2a4e0f753200202a77dbbe8f898da2832307cbde8bbc7f9cfde6860349</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>4fcb2584d8c03ad586b2f6cecde66df80ecc67556a879170dd5698b4a6dbaf44</t>
+          <t>484a7674ee3a2440478fb97f7950342dbce910a9f816a66e3515a2371a93a81f</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>5c40084f3cd60d6990571b279fa8b4b77c770aec6e040941af90411c0f3a6e72</t>
+          <t>66429b419661724a9033230de7a3f8c445733fe3fad05dbcf4ee780c80fac1e7</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>68c0da516f5c569ce1bdcc3843d024949436df69a7e15bebfac391e1cf77279d</t>
+          <t>616a64446f5aa6cf0096dd10df181e389eb52948eb0a9e32a163df2a265a4065</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>0d6a8d74a6804397b39cb4b8accc4f1252d285d9bc6c9b7dabfeacb6d6e902c7</t>
+          <t>fa863a2a05661bedd7cbf677a887f130acd2e2c60e57cc321c491c585959cc4d</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>c39389f958ff509874456e5eb145ca9cc76e5a3cd9b023fb1ffaf7c3b9978544</t>
+          <t>c1624bd67666fdbf4559be47ec1cfded0846d040c2b68f23e36e2fb5c53637a1</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>0d721427318a45c0100cc8964544b42d970a8165fc93f77d5bc92eb648d1436c</t>
+          <t>1d8ec4c4a7691c6f3c42fe02eaa97fd3ff0d92422f3b2d6ea7d90b50161b848f</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>5aecfb32a8520e4182cb78eeb9723c07b63f67090be3543e1e5f74f0857cba56</t>
+          <t>a1732a41e09cdc58c4b2969f99cd1572f9dbab50c0afe8d69f5978053e7f7217</t>
         </is>
       </c>
     </row>
@@ -7472,107 +7472,107 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3551105c748b13450c5b712a09eb8628aa9eb90d782b71c84bf58747002d0747</t>
+          <t>100ef85a3e7a6da1fe99fb27a436d4faa1fe3cb928163c8c9b494580605f9521</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>9ae5e7103b08f406554a6807067d23d23788858ada02b0acb74515450207d91a</t>
+          <t>50c44c2314d62a7ac48e566473f44238e65a6798e628176574e3a8b7c42770c3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>e2df040f1e75fc7f48b3646de6ca1999a73d73d15894050fad35bf310ef6868d</t>
+          <t>900c16849e0ccfe4dcd4dadc495e36377720c6862ba3a1d65b31ae98fdac3f1c</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>04afeec2afe2757d8265cd04e06e898a7ed5d7490e29f673614444788da6a4a4</t>
+          <t>8e92eaba3d69b550676a691834ae6db42d0b839e286c944fef27db92cf709740</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>680e10ffa8eff10f7d5bba499114def4c20e8d09ab88b415a4854a9ed33c353a</t>
+          <t>3c2cab61353a36d7c61b594bc646bdeb0b0a44b882abc57512840022db6208e3</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>523a25b477d3d7289654711700d66e7a130e995734bd86e1130218fd86373ed5</t>
+          <t>a642062b3e287eb8dac3ec87954db6e162017c7f477659bd6f1b7447269a8d21</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ca2f5a1c9322cb6c92c78ad76ba227cd1ae98c47df056ed1cd330c8ae0fe9510</t>
+          <t>a2e4ccd585753d80b83aa50af49dcac9e06938d2e90e33f70e7a567c5cce61cc</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>a7a168ca0cdefcf2668fc4293ffa03c6eb305fc775cc1fd3099dc9a700e0fe79</t>
+          <t>6a4d3b1aab77609de0de69cb56cf419d259f231ab5a7a8854bbe993db1c4572b</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>15291ed43efd604273f0015f7ae1eface98de3edbe54fddac6218e103455ba2b</t>
+          <t>f212f6d985eebe7f8193060fe074bc9622eae35f66241370a3d95a3e569e5d0e</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>f8d16b59384c87995340f48682f601d2f39c13537607e454a2e0827fbdf59e8d</t>
+          <t>ef05b27bc63ac6b5dec642a5ace46cc3ac2cafc9b4dac21c422c0009147cbba9</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0f2a375dbe6c2119a9f4cac832a6fc8167ec0117805d67c85ed05bf129302a1f</t>
+          <t>25d99e73922f4abbabe5b711685a47d6f0cc381cc257321a0c878b7f86cefdad</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>a8e8342d99b06d89eaf2953a854daf371d63f1be5a249bcf821eff96cc6bd5d2</t>
+          <t>da33f29c87db4d87e32a6830318420b21f728a2573c60ba5c57d8f426713336b</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>f6445f0d404d9efe94b4a6bc870e3ab9e82bff9b6a5f4cb1a6c165efffc54674</t>
+          <t>f96ff1e874ea938edce5ba107c9ef179982e0d4a8db0aecc9f7f3e24047b9c02</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>356723fa7c978b119b7fa8ac3d10488be205911dc406aea8d07655a8526d8a0a</t>
+          <t>f2621ea1c5ee56d0352ea5e429fafa59cd5f4b39770f0bb1d35d7b7f282f1fb5</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>1f58897670099d4babc3f6007e1eb4ed21bb855339a04eaf7683f720171c03c0</t>
+          <t>4691cf1bb467eb48dde4354e5640720159d9e1a1eb09861bba8ab54ee64d7371</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1cb4464b7657089766b3162a98cb3da1c8aac547d68e63c5db01c2b1456e036e</t>
+          <t>7aaba8de07530bac662a84a8b91ef1d10c9dad7932303a7be850ae31403b3157</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>83b344d85fb635fe465c1d6c9c3ed53aafa7b5852c30876e8608cd3be30a1d4e</t>
+          <t>eeeff4c4b05e43b0f115a6340fc5578e6a25cefae86ecc8aa55258e7330d3f79</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>ac49125988059cbb1271ac952597a46d4cb37abe7f9a06be46411d58a891163f</t>
+          <t>07c676608b28380d19f47649a2e06dcdf76ea838efc6ae5143840593097e2e12</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>9b927ff63337de57561e842c667186607d3944e8676aec583bac7f790a01dd36</t>
+          <t>a6362898c0e441f965e10e3d8a4c434d170b92a21aad4350bde2a5abf924e350</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>449af92c92cd906c9dcc859eac16dbf853e2f6a345ce3ae021d223e35c2c996f</t>
+          <t>2a73225515be0fbae85e7c6a4dc87f9954e210492ead99a5e8721256a6f72657</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>68bd4aca75097302fcfd7139865a734ad25bc47a29b110feb80a387353df27f4</t>
+          <t>25ac738790dcb450d0c32de620df8e2881e30273418f564fc0bc7fb66390343a</t>
         </is>
       </c>
     </row>
@@ -7584,107 +7584,107 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>d8dfd26a222621436887248b0e75f1217f55150b68f136ce545a4ebcf63f0f32</t>
+          <t>21ad4866962c7734ea2a8a2212a2d4eda45a55258f2325ed8ac47334ed9da547</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>8046d2a888761afc2dd3d408ff06e1e2d5f014bf6ccfa30d4020e6dc9bd56fcc</t>
+          <t>e1bbd00554b5d4692714149cc0ed5f5d1bfcd3b01b6a5571e633fb011d63896c</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3c8e1c6bffa9e6c4c41ad551faacf0e2501c48c5308203eeda0bdedef092fbe1</t>
+          <t>6e1186381250bebe26c94b4f2cbb336621f99ca5078cbf0e35c686c810a272e4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>bb628fcc08fc2ac02e1e182e24b31c8a0ff69c4802fb1d55e6dd44d4b0f25901</t>
+          <t>438c723fb4584e4ab7a7aebd7b5c818fda77a029d4245f6ec0c1013c19569bbf</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>6fdd746034606226387fd1370cfd1966ed5ae0f7c8f914359673941f01423184</t>
+          <t>8140275c8e90bfe64384c6cc2c56b06b078dc60f7e03108db20245db4b41a306</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>448113b891b75365062218083d704372ff568cfb9bf04ec3095c2a50eee7ed3e</t>
+          <t>fac273da676934748dc261127211e9dfc113dddc17f95702eba5733765a48517</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>b88ae4a483b3df146277fc641054b184586d809537b11cdde188be23d155545c</t>
+          <t>b23dcc2d2b5483e86aab6421b09fc923e64a3785b761df7768a651df0186592a</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>f1fc1c57a2a77bda66408b1cca96e515636394a2bcfa9f1169eff7d21e2bd621</t>
+          <t>58ac1911736d17ad099fd90103d6672684b3897ee1709384d51a063b2f90b5ef</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>ef36c5b65057adbfaa587e82da2eb25f3af62ab68d359d1df0aca3dc0d2e665b</t>
+          <t>5ab1e86da0fe16e26fded1de93a26b422081e58e4d033df8ad38ff35f174dbfe</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>cb73413e5b9449b64e8e68e57c905893a0688aded47c846bc4235c03adc17c10</t>
+          <t>f1a962371b6810d219edbfe3ad9725d36c5bb6e16beb85ea41fc8dda585cb50d</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>3a3735e71aed7f372fca48ee6f60d6bd8e2c805ff9e383bc3f44b741839f0a98</t>
+          <t>900132ff358f55ca4bac049716c22afd6853bd9c1d6fd79c7579ab77401974b4</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>88143cd8bbfc5bc18c05aacd74f4c021370c0b8bca1ccb25eff951a9cd482f59</t>
+          <t>831b5a48b19b215afb6e2072c7a717759c6ff895e3b0fef92b2132fef66e98a6</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2744398e758a3aea38b08e8475ac4e461b718008b1feda369107bc9cdb515749</t>
+          <t>41416b2d252926b2b249516514e1c6ec7867443317a10f35292b027a4a8c0cab</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>9d008744346142f8f89e38556bf5001e14c9c5f629dce33686357b6e4a113ccb</t>
+          <t>b8b3f60bf8cc9123db9bd362d3f5dde7abaddfdda3c5408fb997a0bcb714d681</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>77ee1c712bd410933bd027356fb97ba7d2f0a2010be5185ce4106f770e684d00</t>
+          <t>18c88ab9ca747fb93235e471ed29da09a3f40ed6c7b1558eefcc089c71adaf4e</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ed80d00a9e112c3992908dbdb26b157f46d7e4a1c05c8c9545b082e424ff964e</t>
+          <t>550e89fe4f4a2ce0e5d0079a5a6be177c713fc5ac3d4522fbe1e1683da60808f</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>f1a1150773eb0a06b050db6f6464f74428f526cf8bd04a3f486c8d0d163979d5</t>
+          <t>5e07ac1f7817ffeffe6a222c2f1b84fd43b23185006cca5e1ff6b6140127ace6</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>ba7fcefa10f9788b2fa497ad58988bce5cee50848f1bb2297503e7b628f64551</t>
+          <t>6eab3c4171409833ed1a5c756d44f86ffd6621127c8949a8326132fed23d3e81</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>fdf7b3dc55513e821def7ce7e5b7ea8f575fc27e7e64f6af1c5ff4b95ebe9592</t>
+          <t>05afe94d68a1d3b242cb4035a37aa8694d447bbf99f78c58cf8aafee3808212c</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>c78a0921ce05af83b9f156033679568dc890c7fa054c5a3847c6102acd63db3c</t>
+          <t>dcbe2400b48d3593819a09952988b648e9028d6388b8e6e95e30c83f6ffc697e</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>ba515e87fa33dbbe6f44d64f407d6738d90bb741d6d4d7d6b3d1213a1c527da5</t>
+          <t>086761992e6f180a0b006450b5609749ce53861cb1b6ee26f0998aacc5c395f4</t>
         </is>
       </c>
     </row>
@@ -7696,107 +7696,107 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6d6cba5e1aa4d0c0ce3697277a1fab4d4433ab4a2efc442d9cf2f9744d6ee93d</t>
+          <t>6ec4e86078964403de45f546216c2f177351a11e8ed3fff1ee91c4bb5612d3d1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>74b7618cb19570f68880929a616eee84bab13c794ba6e98d135348695255d12c</t>
+          <t>40bc5668360ad677a43e80038156fda24b8e3c6fa4df178045a927387516fef1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5b8d9e0d35fb40b4ff6bd629cad8048c0d851dd7cbc3b1576d59c75a3a3b6873</t>
+          <t>d7c433d8fc2003ceff78cfb56c30268ceb68272f2d2fa3509ec3f9f3ac6825df</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>a2c15f3cd28c667b7bb4407e0c85edc75a57a3e3a65629969dbaee178834fec8</t>
+          <t>2cd2449a9e995223b931d3b8b416cd233717eadcba4ed2afad44abfab6ae6f31</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3b2ee36c01d5d18fdd56a2cc21cef9d4842b9c0b8ba05f47ec4b5e2a45a6ab29</t>
+          <t>af8b742d900f9c3547529e70d4687c3aa37b8b3db159d53bcb1399e6fdac33b3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>837eb913294809298135132b8cd4d5da89c729ed83229a1da7b0a0c4b8d6171f</t>
+          <t>ab16136fbd32762c96e5c14db4d3266b58d25e8bea4a4da5b4a4e6209cf3ec17</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>94f6769e3cb90e4aa931186394743f69ed67d51eae51ba40586119992632b3e4</t>
+          <t>67435ce8663fae1ce448f8d3e4b710e195b169dc7ac747fa025f83a6f42b2d13</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>d125f76c465de551367c74927aaa4c4ff89c85336248658896e002245492e803</t>
+          <t>c2d0fb1ece52204cc4ddbf77c1b1035ad3bca6aaaa154d9e9b8d01d148b59029</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>c2ebef0bbef8ddd4dfa6fe8325bae86b537d3ad0a490af95d03222cb4fdb50a9</t>
+          <t>93301994c0b234b2b9a4d6e8d9ba1ba554c9af091745932570363628a85ff4d9</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>74e9418cbfb67e6cfb95e8f196b8e4ba73b4b80e39d9c07dc1ac620f236253ec</t>
+          <t>1fba705858dc893f836e1707a207eb1e326124a24339cdc1026ee9f924e44512</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2984b61ad8b990fe47248787e2372cdb370341c0b9f8793fa19834721ff8e9d8</t>
+          <t>ee49f499dfcbf811f841a675b66376fa30220445edfad1fb1b6f4f03a567ed84</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>5a7e14fe4ee769b1cc0f640441e5516e40e99f16fe3f0367193f3fdde37e51e3</t>
+          <t>e8712d9e570934f155f743a57054691f5308ca26fb899398072ba9582acf099d</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>ebb2678c43b27a78388264e90f2b3c7010d3079611114f55d5209d5e8410e2d5</t>
+          <t>ada6cddd5a2e1c782fe93bf165f3e7286859322e26cb23b3a51f9c6491d5f67f</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>52757c0cc175dd5286aa71e69f1c61b3ceee165c6041126b39857586b901d321</t>
+          <t>3fc014775c749879eda9bfc854b552f71a80e706684c89f57d2edb7bf75624e9</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>7a1ed27b4a4bfbaadab0c7364d135fcad7cd31e32b238f6bd575dac13f90d77c</t>
+          <t>7fb8d3f2a6b9632d39564f0c925aa4434636a1b0134c4212e040a1df1fc67637</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>d1e19bdf8ceeab830f970eae9d35f32f54fb275cc327b4fa09a3808b438335f0</t>
+          <t>6be1d7236b43af9561cf8d4df84da5ceb2e8dec86b9dc69b8b15a19c3d9fe1ef</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>ff032a2a8bb9ce796af998019fb776bc237b49541fda8c289a9ee245649e8b0c</t>
+          <t>0630a2a67813a23a823b6e038c7963e2b0a6d2ab6a1235a1f73d7aed5fac46a9</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>a77508084841a7cf6c76c9917220321e883f28e1c870e4a71803faca32ddcd58</t>
+          <t>4e67ae96af83cfac08833b06573514ca54e95ce5c38073bcf6b4296b74f7a0c5</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>47e4a4d3c8acb3e1b8a9518d8a7aa640bea3a112cc57d0597ee726540d87a502</t>
+          <t>31fc6330cda16f94b385d21f2684c06c689ea90f3f8a794aef1f3c9b39a5d045</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>95cee1871671cb5536ea2c203246d586b11ae5e38779695b8813f5d2ac18c7ed</t>
+          <t>186876d003266e74c633e904b9ca1298e149d8e032245718c1b7a5c5b6bba010</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>0795035a538488e37a9ed63284a16780f327aaa6af7172e354d7514dda99b1f6</t>
+          <t>0f13ac83221e60ee75738687cf99963dd4a0e07b12223def86140ad9c3b0ba90</t>
         </is>
       </c>
     </row>
@@ -7808,107 +7808,107 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>346230d02910582a26e6a04347a1ad396811adf65ac37a935f651f7ce7951a7a</t>
+          <t>781dfa3959b7336a7958c9ca69d72444675d5662a3d36b709fa4f70d1756d412</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0b5740a67ac913c744e0f8b0952bf154d1b9cd4925fd177d95948bc25c55089e</t>
+          <t>1c0df6356992e5ba212963d049619ff1708dcdcb5fa2b9f2fbe6089ce1b1a823</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>a9d6b1dce195113d11fd6babf896cb2cd3c9c1082317ebc0c2c365108020f4c1</t>
+          <t>8e6b4c3db396bc6b758a04fc2ca2fc2dd0bfd497cdb5e9af4f93d364d8381782</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6170495c83d8aaca4c46a0e6be3f713b2174418d5d38b4745fb831531be28426</t>
+          <t>bf77f666604c5c48d8057e359bcfb9aad31aa1f8ec8368c0f0e6355853abcf0b</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dde20bd51831263fa10fe058f0caf3edd085a855c2782475bde362579cb02b50</t>
+          <t>158792c7a057b664e3a07b61aeefd9f87fc8db692983fe93e7a3b6cf2d8ce49f</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>a0719103832acbbfbe68f33743057c30e75e2cfb409ed144cc3f412bd785132d</t>
+          <t>69387cb37d8f96c084b245405a72b3c0d425a1535bbec3ee85aea9a2709107a2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6cb7165db49d0f2ebda051c7d95e7f55bef9d87ff0e461e2a5516999ec498084</t>
+          <t>9af3fc89ee2fe022508e8fb5f7ba160e2d36f4ab4ffb2067f8ce50491ae3b8a6</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ccc680d031b83e7e7bf9d0c25fef96cd61eb64243061be2339b49102f827072c</t>
+          <t>a3b526fe2b14c82447e873f4b6f711079132c26895dc48367455d514a97acf0f</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>bb171fcbc589ba6d18e0be5650fa8fbea6ccf86dfe25615776ac3ae32cdfc1ae</t>
+          <t>f4e12ebbcdbba01546637003a572f11b14e51e828f0db86663ff76399dc9718a</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>c72840bb4363a47e7492fbdcd6c5a6f6450f27c6d8e0e4f9223dd1455839a68b</t>
+          <t>c00afa18875c5cc79c4579dfd0887a815912a4c2122a53fa0cb834dbbcf325c1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2cbdecb513feaeefe5f92e4732e33375203f2e53ee6a987b5f301ec5a56e66de</t>
+          <t>b9d92008668fc5b17b9aec0fdd7fead2b773a9e9d519341505d7247170e1c039</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>c8909b57d5695bcc2ebbeea506dbaf1ddfa69653c854fdd00176eb8d1cfcfef0</t>
+          <t>31dfabb1dd79b5d61b025f41db6afe2b6f80ffdd67d01ef436f02039fbf99b35</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>4db15d4f72c4e4d2daad79e9458360b427ea71d3eeeda8771ede136e6e77afe9</t>
+          <t>0a3c88db7bc765e1764761391fd3395e5fb457e357434cbb2706c3a17c1b0daf</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>7cb93ec8b2b4a3a92ca03abc75a566110acb004df41b4e321651e65c0cf001e8</t>
+          <t>2c6a1a3d799eb03275a07c4cbd01ed193641c8bf8b09f40ef514aa0cf142234e</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>d775db78179ef3318274e177f3898f0919b1d74e320475776be33e25f47a248c</t>
+          <t>03f97eff6be37174077f927c5f29c9ca85c4c8b801726fb801281893995b2705</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>6f42bcd9e96661068c747f67296f0ae633d8c1d059de48b9ebc9a686ac56e5c4</t>
+          <t>a8bac977506fcfddb1fd3df9e1233ecfe50083fff618ab91cccd3d6eb39f80b7</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>fc0670f242a2d0ba0be40420072d7b5a3de5cb809fc74c5593cdc6dab91f2ce2</t>
+          <t>507d7fc54063b245406e5278603f059a23a9ced8742f349d0ce592d965334b8f</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>d3cf4f514a73132b1c424600e313d24aa9d65190d12dbe9e24bd22d14f6e955a</t>
+          <t>4b2c5064f34ae7d255f325e9cb295325d0c3e451a6bc59d70e7d71e4d3622639</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>35ff865dbe27fb9fdf4bb8b8d0923e7bc5c512d36e461fe77ff61c51656ccc3d</t>
+          <t>629885f7b90650347a0b73e042e13a0e1c42522979dd6adaa893ca0fabacf201</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>65e7cab80ec9a9bef7147b189edc448a4a637e0d288ff98ac3f9b94e850429f2</t>
+          <t>5c820d04e0193c81d4a44fac0c9bd39d27dc9b57a4cd101684d14803bf2be241</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>fb0ee62a19df527497d77da3934ea1cd66a1c1532ab926b893d1c05e6b989913</t>
+          <t>863baeec56688da5406e6dcad16ca66d3dc9b8cd512a0b415240a267367a3aed</t>
         </is>
       </c>
     </row>
@@ -7920,107 +7920,107 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>8723e3d43a761dd0545dea18f473f57c83728c798641e8f7715303f77e70edf3</t>
+          <t>82add7ea4de7d9232bcf14c10e5cea48fd0ad1d260109050804d0a60fa8d8386</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>6fea1ace2f20b1f1c4508ba9b4e14968c307702449f2397a58166e6ffe60b17b</t>
+          <t>18efc47e062651fb25065cad67af78ad7ba8653c982fa8e052cf90aa5785b218</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47c00cee2dd71d4ce0b1edae017dc9f9a9c83d0bb22b86292918f3e8f632fc0a</t>
+          <t>27fa86751aec9992b82f146cf395b4f769b0a178dc79f5847343bef44495f47d</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>c54e5bed497b6bdd0f2a80b87a87d079ac6ec80ad60adfb70b5d2213ed0e1080</t>
+          <t>b37f3f35880ebfed8b14298de62dd8bb550cfe14ea72f02dfa2088e8f8721884</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>b50f1f6819323d5f6cb6d31271b557b39acb16897484f645036ba816380902fa</t>
+          <t>1f61ecb739dd2c0a1d2e4e7f1310f328d6c3d434670254fb70579fec51b92a52</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>a8bf9c98bd0d2b798a54a42e74ecaeae8bf7a90938f9f39591f375947d8c9933</t>
+          <t>27a51292a419f1037d1740c1bea297a68dab65d1d0c1179659f88683dc082d7c</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1d3054f567d00ca6f9d15872cdd045aa6ff1b5ca943549eb0a2fb8d062a56c30</t>
+          <t>10be88a9f54c556a9744ed5d02aab5a5aae63e55a889acf5ffe715ea81ead1e0</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>259fe73eb7d2798e830e46be198c86a61c3638fc084b0f68016914e325f16172</t>
+          <t>fa51dd12cb27a91f94b7ab1221eda430592ec87cb8af4be909ae625922641859</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>bbee4bb2d41dbc0b3f4596783925d44ea516e40e563af0757764720430c50d06</t>
+          <t>cd65f2840f892a1f0a264a4e84f0070f2076d2456cfc9afa4887a56ac82085ba</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>406f98a588bd69c00e6e689c251aae52f74f5acf1ab618581b998b9e7a5294cd</t>
+          <t>95b190e3bd23e2964fa54fd065d5d190b8af79626668d61f4795722b2d70b1a7</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>6cc97f45a1568e85fab5b18a9ca5dc479237b4ef68850d768a0d9b87b75df0e2</t>
+          <t>a9fe9e1bff8d71be47f7bbf78b5592942d1f5ba778e9ff85f61f73a405cbe721</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0fcf4dc9ce99c97b3a74ccb0b2aeae2258c6f1e53ca6a0d89199447d7a87a933</t>
+          <t>fdb8af8f2a5a798443bc490caf3ebfe26a5e936e3ba69d4fe8e309af34cd8b67</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>a62237efde7d0cb32058c064155d248132d205af1097c785e1cf2a5ad48b97bb</t>
+          <t>2e75e6d3801818cd3f4ae303fae558dca1e50d880664f41e40701014f2ee4432</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>5169a30798aa365b0bda7587d713f672c7a5b68fd2fefc6204c5f0cc4a61e352</t>
+          <t>bb82a9caee2ec843fe90c025a38dc1aca612a9b1bcce97088ebe2a76a480e49f</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>af351044fb55892d9c305253c897b92118159f65d096f4377a8f061cf681aff6</t>
+          <t>83bf10327ed4ca99a5a57ad6f8e1589d85d19b9236ddd5954db915a18d0aa642</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>65b9631d2386304988d3798e6482c6c76fe29edade24aba3145a8bcff9da5eba</t>
+          <t>845d0d1d615ea5492f0dc2a343df25890b8445076640ff1ed8a2c069a4c6c8c2</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>60d4c445c9ed615d3c64e5430b54606d1dc110938f4eef234a606169191d9fcc</t>
+          <t>57d546db009c93e66ada2f61be975441e126a2b34b95499cc02fd738cfbc6cea</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>3e5d6598e0fb857689c104d079e223e252b769470a51694f3870173b70edc03e</t>
+          <t>d59305ffd8143c18a53001696f994a5b88a18a1fe635ea192a85757d7796ac6f</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>12640e2c3aea7673436d7766a2da3a61e2f70cfc239d108beb6c7b3b05562306</t>
+          <t>5cf091aa7ebf48f843010061f4ef363a491d1f60597e6877c125f3367302bcce</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>f030db39dad551d1f0e6c9166369074fb49c3843de9cc1dbac5cf28b486c2f02</t>
+          <t>254b405355f45eccf8bfb50c287d154bcaae0f1db6d2ac03da65cf05b7083409</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>ffac5bf972317ad85a9eec2f72e3c841645a9d0b6d38f63fdbfd28f018a9ef17</t>
+          <t>6b7f7fa6cc1c26e6ccffe83a9f4632ca07350b3a032156f7267186e07ac67e4c</t>
         </is>
       </c>
     </row>
@@ -8032,107 +8032,107 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>22fb61188e7856d2a50c7e42b6c9b3065c0c2e1051abe5dfc7c075c8b4e0c9c6</t>
+          <t>02e646ce1bd822df9554ef8179ff3a73d1abc1729e61e67fe56a412a95fbcc5c</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>91bb4ca854d0ee8122e5f4c9fd3053640a7006fe378d953228a4d4ff0701e4eb</t>
+          <t>18809f58569e8cc695a4864ce760c26e45e3f404f939b7ed6c500f1590c2faa0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6ceb34030677f6f00f71a2eab140b67420f58e225b503938e529d5dfd60ab5c8</t>
+          <t>04e43fce95e5f7da960dec31e1d39cb770808ea673585eaa2201f90bdf5bec4f</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>b685d1b16165463e14fb9a475f1471856db17449190ca5d31ea6ea8ef8d5c5f1</t>
+          <t>df227e7f8f5384bbe8ec7e3e69dabdb22de894084e38ed976c99b84d9fb9e9c0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>edfad3278246baddb625b90fed5edca12df83550c6638f275155f459e1358be8</t>
+          <t>b91396bb793acd3a738f98d93d493f01ec5259c4b98a660f8b7b1e012fcd66c6</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>b803256d652976ddefc2548b2374b0e77061805b15d17c79e8df290cf01a0ba4</t>
+          <t>9d73e09cafd0e91d69eb045fec1ece8bc2b5e512cd2b2822c49f641b23ff52f2</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>de76970b1f1bc01fadeda309eb2b28fcdbeaf7dbe159cf714ee8d537da60c488</t>
+          <t>9ea1587b7f6e90adf67b8eb3923795c9c17322f1e5ff122f1cede7dfdfe74815</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>05d4ac1f38a16dc2a0f3b8b2fb1d4789bbee4ca79e9d02892cfd446578d2bd8b</t>
+          <t>45e7578f3392005709ca5163c7c17609ff333ab1575f65d8ae05469b5f98374c</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>f16b3cfb4990495524fe77cfbff0c1e99885e020bd9c0aacf6733ed9f39fd0c9</t>
+          <t>1b67f338dd1dff5a1b9b5a7f7cfea7d8b54b946710fae79697b416adb5dcb520</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>af6f452e53707b1a39bd7855962842c082f1d574399adf3359e3b652511aaffc</t>
+          <t>38e6b480d96db447320a8ea1196c6139d3d356267251b24264359dcd3225a06f</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>b9e570ca851d06fb3ff134e592309ea3c7685749bbb420822fce6cbab9d75d5b</t>
+          <t>fda35a4d8ab497159fde5abe5d185b87e3c957638b3b8876948b2b5f05e600d4</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2415555df93672f2b1e5851d7d17bd364d2c5c387bffc9c6d63932fb16007e79</t>
+          <t>3e9f5afbb851f29ce16c70fe28fd732026f0250defab221a5152ace170cb540f</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>df977ce2e219e3c294b1407dfb8140b5ce48c12789a3136751e05e0cf8deaf0e</t>
+          <t>871d2de265429d202ef4d85d0650ff8d5173f2d3cc97f96a875cf10525600f29</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>0bbfb46f7955f6c0e8f33f4cb7338ad3268320082ecd3bf942092272c6cca6d9</t>
+          <t>29f60a2275b3943661591f05eb31d71852572b69e098f303da910f420435c400</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>ec0e2d0b1d26059f7866fa81cc16b9a2473c0bcf26bb1a2e7eec2ba171515a27</t>
+          <t>c6ca84821e117aaa4c18d3c3877ab3810811a0d1236ac899eb4d183f689f5e87</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>9d4bbe4f9227c65fea96dd1d93b4ac0e57cbbfb8d03d105dbb7ba08d8a673602</t>
+          <t>eda915e49268c74f5b6ee56b88c83d7f6e652ffcedfe08d40813d79d3c195704</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>a63ef3f5a8460af145df9efe48637d891f5a9031bdb6f2f74c229ba799a0908e</t>
+          <t>f1f3d55632d950c0af34fb53897eabb4a9ffeac62e474c11d8710e1ea7869334</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1b58f16c95a8f0d496cf30703f31f94486239d2039c678fe033ce0f3a8301d3e</t>
+          <t>4f602e92bbee93f3485b6a8aa55eca6f52ccbfbc18bd854d17a7815537cbc895</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>6c962b232e58f0932d5b3675e256d2e31383311f2816cab5b53b7779eab73fcf</t>
+          <t>67d7b415b1516ab4f69b1fb89c539f07f6c70f8be06c1cf6b49792059960eb64</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>4d788da0d861cf4deabd0d4953355336eedf0f0857d25bf04b9713847684fd52</t>
+          <t>6f74378d9c67a5e8ae05a503526349807377fb2e404e0cda1cb9582399248ff2</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>a98b2d158d82d34521e01a95c7fef440a20719ee6569b9da52ca44c1e367faae</t>
+          <t>1eb3ef9c6eb909b72bb01c67cc63ca46ef8d2caf369b3bb00b9c476dfbdb8fe5</t>
         </is>
       </c>
     </row>
@@ -8144,107 +8144,107 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>e3f96a644a5f7da643ea99f126cd3ecff39cff97d5c89213c51fbf012468e0b6</t>
+          <t>e20ac8d07bddd3adccaf890d6b6c081304d1d9a9725b34342583f336ec98f247</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>c9736b0f91f7d1529636db3fa3bae743fc46ec05c0897e4d8920259effbe2fcc</t>
+          <t>fc7fd6f1f354f7020316b671ba6cfaaecf1a6501c6024e8216b8c87e38b4ab20</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>e3bfe58be5ae40aaab3ef0e09ece58b00e65e6b389257ef989a3924e5b765755</t>
+          <t>53dff3a20dbafdfb74d80930704c802386ac1a3d1e903d3aaad34265222872be</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>39b8993e4478e4fdebcb63a6820fd580b323ee5b037a5d171dd83ca4d56ea809</t>
+          <t>d4a101ed66aac4a22ab601bd28a6098cd789317f327234ad18b9b54ac844adb5</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>4ca7d741cc776e3e817646a6dd4782b84a3ac2b22812e4c990c59e52082499af</t>
+          <t>d56953da4985173675f3a1c0a58e2d59d3f378ecca3684519ba8073bbdb5dda5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ef95f540db3143ffa9ff5083ca19144895cbc1954693290be2fa1f01c6b3ee34</t>
+          <t>34b6418b684cd5752f44938050264416f095a6865bfbc7c5c6be52682704375e</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>65c87570caa375a06c52036127b26bb5e2574e4eedfbb5327968b680312b4d47</t>
+          <t>c406ac8fd6b27bed2cc9f504256da3666e688231c5b3cee6f6081b8dfc37f13e</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>d9ee887b8378dc20f8b5779ca2b0b4b14ba7b3a5d4b76aac783bb3e75e5a96c6</t>
+          <t>f8ed4c097278c1c94d4c97b10734ba0173c85fd0cabb5c652ae714bb32638d99</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>322f956b54e7a8c2e69a1df32e320a6b193903c210543c11132202de27d4ac31</t>
+          <t>a35d72367930bf1f53f69e1ad12078f920cb21d67bb1b00ec35a391ba42d657c</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>9c52d9ecd6c41737cc1369026c746c534778a73655f656dfa1e786492416164d</t>
+          <t>09c3479ff2e1ea999370d2fc86c707745b88605aaaad9f913e8b87bdf70ad178</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>f2350adacf23ca3de06ad05822b0ec0eba759e80ed2dafc710bd2e9d50975f32</t>
+          <t>93229e193d2076216327d67cbca14f57c28144964be6b6a7827ed8d607911af8</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>11db1d395b7a1d34057ebf6bdce19759b00b8fbb8555f5cf5391a56b88c73379</t>
+          <t>10731aebae3797ffeb27bc7016ac95915cc05c918ecb10e79959487c8c0f028f</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>7e79b18386c563ea520f3ae7a8beec3afc6131b7e53aeab54934122a9147a23f</t>
+          <t>db94c7849637f956eb94a31e14e92bd3d9f52ab1fc870c6918ba56aefa3da2c4</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>5684eebf77196e48cf7bc07677a1c365d72036094256c8496e42e4c5a876c4fb</t>
+          <t>4b635b8a4257da26194951d56892501cf7d704605bdcac33a717ed3b54bb7d05</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0db08638d16faa8bace3525a07012cd542e56bc9f13bb50bd859afe475c954a2</t>
+          <t>906c7055b0cfb07e5b638ea6ace183157c7b2e01f05067dea7012334e5f588ed</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2cf6c3e29239b7e0eccf70609fb6e9e99c7197988cb42755dbb5fcd888104ae1</t>
+          <t>e42cc30d9a33427d754293600301a12002f66bea3e4af5a671fa6b622bc52521</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>b3e7ea10667e5b2b49d602c4d19971c13f21c19f16caac73911e77d71c515eab</t>
+          <t>7858c2a22fb91687c48b31b2760334ca686d4715795307a9e5c9e619696e2322</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>dd2a122535ab4df6fcc4423c3260ab43cb3faadfe03b2126553fc4c80e34fa91</t>
+          <t>6ff8309a65c50e1676c8998e435f0312a634df0a60aae662e3256b1a28ceccea</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2766a8732d0dab45268024932580d8b2ddfd707cf57cdbbe891b86768ba5089e</t>
+          <t>3d36df7f84c4146d4913e57f3a1df08f9b17840d4d30bb0032b8af4743fb23aa</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>cef4a00793bb9a641cf8852de39100e7dce1d887932ea10ee8c0a0345435ec37</t>
+          <t>0486cf36df5dac3146631d25af1d9ebd3c89c79adb6ae149e28ff0c8f5a3ebdb</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>30c9cae772372553c38c674861c43549d1a0ca61b313e89295c42a12a535cbb8</t>
+          <t>15f76bb34a57bb3c12d526244610c89d466d180e20ac464349c84666ba22054f</t>
         </is>
       </c>
     </row>

</xml_diff>